<commit_message>
added matched-vs-non-matched plot to index.qmd and contingency tables to analysis script
</commit_message>
<xml_diff>
--- a/data/raw/data_articles/v10/datajournal_articles - analysis of citations v10.xlsx
+++ b/data/raw/data_articles/v10/datajournal_articles - analysis of citations v10.xlsx
@@ -9995,14 +9995,20 @@
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
+  <documentManagement>
+    <TaxCatchAll xmlns="a0e84d40-090a-490d-8a02-2942ffba970a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="aaacefca-f467-416c-abd0-2b181dff1e20">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100029FD0B41DD07841BED16965712E158C" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e0f1011f30fef6dde8223745cec2fc96">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="aaacefca-f467-416c-abd0-2b181dff1e20" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4d5cb4cdee1db726a521ed27371901b5" ns2:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100029FD0B41DD07841BED16965712E158C" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ae6d51e96c8c66a8de8dfe8311f95192">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="aaacefca-f467-416c-abd0-2b181dff1e20" xmlns:ns3="a0e84d40-090a-490d-8a02-2942ffba970a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f9e171e4f7fb14517da8847a2c60885" ns2:_="" ns3:_="">
     <xsd:import namespace="aaacefca-f467-416c-abd0-2b181dff1e20"/>
+    <xsd:import namespace="a0e84d40-090a-490d-8a02-2942ffba970a"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -10013,6 +10019,12 @@
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -10042,6 +10054,50 @@
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="14" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="2375ea7b-1eef-4e91-915e-32e4cb5a9c34" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="a0e84d40-090a-490d-8a02-2942ffba970a" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="15" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b1b93042-dae5-4a91-aee7-e8b26f1570c8}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="a0e84d40-090a-490d-8a02-2942ffba970a">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -10152,5 +10208,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9EF39AA2-F2C0-4EDC-A7C4-5860D6EF0AEF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{94E7268E-1623-4EA2-83B7-BCA436F5E444}"/>
 </file>
</xml_diff>